<commit_message>
Cargar expensas BONORINO agosto 2026 ($222.825) desde comprobante MP.
Período agosto · pago 01/09 · Op 175716187231. Espejo en Expensas Consorcios
y catálogo MP. Pendiente: revisar Gmail para meses faltantes (ene–abr, etc.).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -665,7 +665,9 @@
       <c r="J5" s="5" t="n">
         <v>209393</v>
       </c>
-      <c r="K5" s="5" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>222825</v>
+      </c>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
@@ -1403,16 +1405,44 @@
       <c r="J10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="A11" s="9" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>222825</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Transferencia Mercado Pago</t>
+        </is>
+      </c>
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Op 175716187231 · CUIL 30536004005 · Banco Comafi · Original 222824.05 · ceil · período Agosto</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>

</xml_diff>

<commit_message>
Completar expensas BONORINO abr–ago 2026 desde PDFs del consorcio.
Realinear períodos a la liquidación (no al mes de pago), cargar julio
faltante ($214.582 ceil de 214581.05) y archivar PDFs en BONORINO/_inbox.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -655,15 +655,17 @@
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
+      <c r="G5" s="5" t="n">
+        <v>200340</v>
+      </c>
       <c r="H5" s="5" t="n">
-        <v>200340</v>
+        <v>219145</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>219145</v>
+        <v>209393</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>209393</v>
+        <v>214582</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>222825</v>
@@ -1167,16 +1169,16 @@
           <t>Transferencia Mercado Pago</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr"/>
-      <c r="H4" s="10" t="inlineStr"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Op 159022197576 · CUIL 30536004005 · Banco Comafi · Original 200339.05 · ceil</t>
+          <t>Op 159022197576 · CUIL 30536004005 · Banco Comafi · Original 200339.05 · ceil · PDF liquidación Abril 2026</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Abril</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1213,12 @@
       <c r="H5" s="10" t="n"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Desde extracto MP CIUDAD (ceil)</t>
+          <t>Desde extracto MP CIUDAD (ceil) · PDF liquidación Mayo 2026 · recibo pago 05/06 TOTAL 219144</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Mayo</t>
         </is>
       </c>
     </row>
@@ -1251,18 +1253,18 @@
       <c r="H6" s="10" t="n"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Desde extracto MP CIUDAD (ceil)</t>
+          <t>Desde extracto MP CIUDAD (ceil) · PDF liquidación Junio 2026 · recibo pago 06/07 TOTAL 209392</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
-        <v>46132</v>
+        <v>46240</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1271,34 +1273,38 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>LUZ</t>
+          <t>EXPENSAS</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Edesur</t>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1685</v>
+        <v>214582</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Factura digital Gmail / MP</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>3932799</t>
-        </is>
-      </c>
+          <t>Transferencia · PDF recibo consorcio (06/08/2026)</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="n"/>
       <c r="H7" s="10" t="n"/>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="n"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>PDF liquidación Julio 2026 · FORMA DE PAGO 1er venc 214581.05 · recibo Nro 00052345 pago 06/08 TOTAL 214581 · ceil</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
-        <v>46160</v>
+        <v>46266</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -1307,34 +1313,38 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>LUZ</t>
+          <t>EXPENSAS</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Edesur</t>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>1441</v>
+        <v>222825</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Factura digital Gmail / MP</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>3932799</t>
-        </is>
-      </c>
+          <t>Transferencia Mercado Pago</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="n"/>
       <c r="H8" s="10" t="n"/>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="n"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Op 175716187231 · CUIL 30536004005 · Banco Comafi · Original 222824.05 · ceil · PDF liquidación Agosto 2026</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46192</v>
+        <v>46132</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -1352,7 +1362,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>2198</v>
+        <v>1685</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
@@ -1366,11 +1376,15 @@
       </c>
       <c r="H9" s="10" t="n"/>
       <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="n"/>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46237</v>
+        <v>46160</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
@@ -1388,11 +1402,11 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>2074</v>
+        <v>1441</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Factura digital · vencimiento 03/08/2026 · cliente 3932799</t>
+          <t>Factura digital Gmail / MP</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1402,11 +1416,15 @@
       </c>
       <c r="H10" s="10" t="n"/>
       <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
-        <v>46266</v>
+        <v>46192</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
@@ -1415,46 +1433,74 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>EXPENSAS</t>
+          <t>LUZ</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Expensas — Cons De Prop E Bonorino 82</t>
+          <t>Edesur</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>222825</v>
+        <v>2198</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Transferencia Mercado Pago</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="n"/>
+          <t>Factura digital Gmail / MP</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>3932799</t>
+        </is>
+      </c>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>Op 175716187231 · CUIL 30536004005 · Banco Comafi · Original 222824.05 · ceil · período Agosto</t>
-        </is>
-      </c>
+      <c r="I11" s="4" t="n"/>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Junio</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="9" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>LUZ</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Edesur</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>2074</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Factura digital · vencimiento 03/08/2026 · cliente 3932799</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>3932799</t>
+        </is>
+      </c>
       <c r="H12" s="10" t="n"/>
       <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n"/>

</xml_diff>

<commit_message>
Registrar Metrogas BONORINO cliente 30010713734.
Mapear en utilidades_cuentas, reglas y fila GAS del Excel BONORINO.
Sin facturas/pagos locales ni Gmail para este cliente aún.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gastos 2026 — propiedad independiente · Edesur = LUZ BONORINO</t>
+          <t>Gastos 2026 — propiedad independiente · Edesur LUZ 3932799 · Metrogas GAS 30010713734</t>
         </is>
       </c>
     </row>
@@ -721,9 +721,21 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Metrogas — cliente 30010713734</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>

</xml_diff>

<commit_message>
Cargar Edesur BONORINO septiembre desde Gmail ($154 + $2009).
Facturas digitales cliente 3932799 · venc 02/09 y 30/09/2026.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -711,7 +711,9 @@
       <c r="K6" s="5" t="n">
         <v>2074</v>
       </c>
-      <c r="L6" s="5" t="n"/>
+      <c r="L6" s="5" t="n">
+        <v>2163</v>
+      </c>
       <c r="M6" s="5" t="n"/>
       <c r="N6" s="5" t="n"/>
       <c r="O6" s="5" t="n"/>
@@ -1515,28 +1517,92 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="9" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>LUZ</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Edesur</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>154</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Factura digital Gmail</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>3932799</t>
+        </is>
+      </c>
       <c r="H13" s="10" t="n"/>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="4" t="n"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Gmail Factura EDESUR · vencimiento 02/09/2026 · cliente 3932799 · BONORINO ESTEBAN 82 · original 153.16 · ceil</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="9" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>LUZ</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Edesur</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>2009</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Factura digital Gmail</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>3932799</t>
+        </is>
+      </c>
       <c r="H14" s="10" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Gmail Factura EDESUR · vencimiento 30/09/2026 · cliente 3932799 · BONORINO ESTEBAN 82 · original 2008.89 · ceil</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>

</xml_diff>

<commit_message>
Guardar datos Metrogas BONORINO: medidor 25767970 y dirección.
Cliente 30010713734 · Av. Cnel. Esteban Bonorino 82 1º 005 en Excel,
utilidades_cuentas y reglas. Sin montos hasta factura/pago.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gastos 2026 — propiedad independiente · Edesur LUZ 3932799 · Metrogas GAS 30010713734</t>
+          <t>Gastos 2026 — propiedad independiente · Edesur LUZ 3932799 · Metrogas GAS 30010713734 / medidor 25767970 · Av. Cnel. Esteban Bonorino 82 1º 005</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Metrogas — cliente 30010713734</t>
+          <t>Metrogas — Bonorino 82 1º 005 · cliente 30010713734 · medidor 25767970</t>
         </is>
       </c>
       <c r="D7" s="5" t="n"/>
@@ -1104,6 +1104,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Metrogas · Av. Cnel. Esteban Bonorino 82 1º 005 · N° Cliente 30010713734 · N° Medidor 25767970 · (cargar facturas cuando lleguen; mes = fecha cobro/vencimiento)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cargar Metrogas BONORINO PDF 280003529220 ($8.277 ceil).
Liquidación 8276.79 cubierta por entrega a cuenta (total a pagar 0).
Venc 07/09 · cliente 30010713734 · medidor 25767970 · Septiembre.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -746,7 +746,9 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
+      <c r="L7" s="5" t="n">
+        <v>8277</v>
+      </c>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="5" t="n"/>
@@ -1107,7 +1109,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Metrogas · Av. Cnel. Esteban Bonorino 82 1º 005 · N° Cliente 30010713734 · N° Medidor 25767970 · (cargar facturas cuando lleguen; mes = fecha cobro/vencimiento)</t>
+          <t>Metrogas · Av. Cnel. Esteban Bonorino 82 1º 005 · N° Cliente 30010713734 · N° Medidor 25767970 · mes = fecha cobro/vencimiento</t>
         </is>
       </c>
     </row>
@@ -1612,16 +1614,52 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
+      <c r="A15" s="9" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Metrogas — Bonorino 82 1º 005</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>8277</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Entrega a cuenta (factura saldada · total a pagar $0)</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>30010713734</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>25767970</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>PDF 280003529220 · TOTAL LIQUIDACION 8276.79 · ENTREGA A CUENTA −8276.79 · TOTAL A PAGAR 0 · emisión 26/08/2026 · venc 07/09/2026 · período liq 27/06–27/07/2026 · PERIODO 04/2026 liq 1/2 bimestre · ceil</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>

</xml_diff>

<commit_message>
Fix BONORINO Metrogas: invoice total a pagar is 0
PDF 280003529220 is already covered by entrega a cuenta, so remove
the $8277 September GAS expense from the workbook and catalog.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -746,9 +746,7 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n">
-        <v>8277</v>
-      </c>
+      <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="5" t="n"/>
@@ -1084,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1109,7 +1107,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Metrogas · Av. Cnel. Esteban Bonorino 82 1º 005 · N° Cliente 30010713734 · N° Medidor 25767970 · mes = fecha cobro/vencimiento</t>
+          <t>Metrogas · Av. Cnel. Esteban Bonorino 82 1º 005 · N° Cliente 30010713734 · N° Medidor 25767970 · PDF 280003529220 TOTAL A PAGAR $0 (entrega a cuenta) → no gasto</t>
         </is>
       </c>
     </row>
@@ -1614,52 +1612,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>46272</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>SERVICIOS</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>GAS</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Metrogas — Bonorino 82 1º 005</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>8277</v>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Entrega a cuenta (factura saldada · total a pagar $0)</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>30010713734</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>25767970</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>PDF 280003529220 · TOTAL LIQUIDACION 8276.79 · ENTREGA A CUENTA −8276.79 · TOTAL A PAGAR 0 · emisión 26/08/2026 · venc 07/09/2026 · período liq 27/06–27/07/2026 · PERIODO 04/2026 liq 1/2 bimestre · ceil</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Septiembre</t>
-        </is>
-      </c>
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="10" t="n"/>
+      <c r="H15" s="10" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>
@@ -2705,18 +2667,6 @@
       <c r="I102" s="4" t="n"/>
       <c r="J102" s="4" t="n"/>
     </row>
-    <row r="103">
-      <c r="A103" s="9" t="n"/>
-      <c r="B103" s="4" t="n"/>
-      <c r="C103" s="4" t="n"/>
-      <c r="D103" s="4" t="n"/>
-      <c r="E103" s="5" t="n"/>
-      <c r="F103" s="4" t="n"/>
-      <c r="G103" s="10" t="n"/>
-      <c r="H103" s="10" t="n"/>
-      <c r="I103" s="4" t="n"/>
-      <c r="J103" s="4" t="n"/>
-    </row>
   </sheetData>
   <autoFilter ref="A3:J103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record BONORINO Metrogas September as $0
Keep the invoice visible in matrix and Detalle with monto 0
(total a pagar $0 after entrega a cuenta on PDF 280003529220).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -746,7 +746,9 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
+      <c r="L7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="5" t="n"/>
@@ -1612,16 +1614,52 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
+      <c r="A15" s="9" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Metrogas — Bonorino 82 1º 005</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Factura digital · total a pagar $0</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>30010713734</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>25767970</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>PDF 280003529220 · TOTAL LIQUIDACION 8276.79 · ENTREGA A CUENTA −8276.79 · TOTAL A PAGAR 0 · emisión 26/08/2026 · venc 07/09/2026 · PERIODO 04/2026 liq 1/2 bimestre</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n"/>

</xml_diff>

<commit_message>
Set BONORINO Metrogas Jan–Sep to $0 pending invoices
Only Sep has an official PDF (total a pagar $0). Fill prior months
with 0; leave Oct–Dec blank until future bills arrive.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -738,14 +738,30 @@
           <t>Metrogas — Bonorino 82 1º 005 · cliente 30010713734 · medidor 25767970</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L7" s="5" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Fix BONORINO Edesur July using invoice due dates
Reassign LUZ months by vencimiento so July gets $2198
(due 02/07/2026); cascade May–Sep accordingly.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -698,16 +698,16 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n">
         <v>1685</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>1441</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>2198</v>
       </c>
-      <c r="J6" s="5" t="n"/>
       <c r="K6" s="5" t="n">
         <v>2074</v>
       </c>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
-        <v>46132</v>
+        <v>46147</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -1414,16 +1414,20 @@
         </is>
       </c>
       <c r="H9" s="10" t="n"/>
-      <c r="I9" s="4" t="n"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Gmail · vencimiento 05/05/2026 · original 1684.71 · ceil</t>
+        </is>
+      </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Mayo</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="n">
-        <v>46160</v>
+        <v>46175</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
@@ -1454,16 +1458,20 @@
         </is>
       </c>
       <c r="H10" s="10" t="n"/>
-      <c r="I10" s="4" t="n"/>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Gmail · vencimiento 02/06/2026 · original 1440.46 · ceil</t>
+        </is>
+      </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Mayo</t>
+          <t>Junio</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
-        <v>46192</v>
+        <v>46205</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
@@ -1494,10 +1502,14 @@
         </is>
       </c>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Gmail · vencimiento 02/07/2026 · original 2197.55 · ceil</t>
+        </is>
+      </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Julio</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1546,11 @@
         </is>
       </c>
       <c r="H12" s="10" t="n"/>
-      <c r="I12" s="4" t="n"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Gmail · vencimiento 03/08/2026 · original 2073.74 · ceil</t>
+        </is>
+      </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
           <t>Agosto</t>

</xml_diff>

<commit_message>
Add BONORINO AGIP ABL service for partida 1084069
Register the partida in rules and catalogs, add SERVICIOS/ABL row
to the BONORINO workbook and Sheet. No paid cuotas found yet in MP;
AGIP public view only shows upcoming Oct cuota ($28.214,40).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gastos 2026 — propiedad independiente · Edesur LUZ 3932799 · Metrogas GAS 30010713734 / medidor 25767970 · Av. Cnel. Esteban Bonorino 82 1º 005</t>
+          <t>Gastos 2026 — propiedad independiente · Edesur LUZ 3932799 · Metrogas GAS 30010713734 / medidor 25767970 · AGIP ABL partida 1084069 · Av. Cnel. Esteban Bonorino 82 1º 005</t>
         </is>
       </c>
     </row>
@@ -774,9 +774,21 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>AGIP ABL — partida 1084069</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
@@ -1125,7 +1137,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Metrogas · Av. Cnel. Esteban Bonorino 82 1º 005 · N° Cliente 30010713734 · N° Medidor 25767970 · PDF 280003529220 TOTAL A PAGAR $0 (entrega a cuenta) → no gasto</t>
+          <t>Metrogas · Av. Cnel. Esteban Bonorino 82 1º 005 · N° Cliente 30010713734 · N° Medidor 25767970 · AGIP ABL partida 1084069 · PDF Metrogas 280003529220 TOTAL A PAGAR $0 → sep=0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cargar boletas ABL AGIP por propiedad según Gmail y partidas.
Los mails de emisión digital solo cubren partida 3977389 (CIUDAD).
Corrige partida canónica, saca ABL de OHIGGINS mal cargado en CIUDAD,
completa Mayo/Agosto/Septiembre CIUDAD, Agosto/Septiembre OHIGGINS y
registra BONORINO partida 1084069 con boletas Oct–Dic pendientes.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -19,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -136,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +155,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -550,7 +552,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gastos 2026 — propiedad independiente · Edesur = LUZ BONORINO</t>
+          <t>Gastos 2026 — propiedad independiente · Edesur = LUZ BONORINO · AGIP ABL partida 1084069 · Av. Cnel. Esteban Bonorino 82 1º 005</t>
         </is>
       </c>
     </row>
@@ -717,9 +719,21 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>AGIP ABL — partida 1084069</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
@@ -1064,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1082,7 +1096,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BONORINO — Detalle de gastos 2026</t>
+          <t>BONORINO — Detalle de gastos 2026 · AGIP ABL partida 1084069 · Av. Cnel. Esteban Bonorino 82 1º 005</t>
         </is>
       </c>
     </row>
@@ -2518,6 +2532,135 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
     </row>
+    <row r="104">
+      <c r="A104" s="15" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>ABL — partida 1084069 · CUOTA 10/2026</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>28215</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>1084069</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>1084069 · ceil desde $28.214,40 · 1° vto 14/10/2026 · 2° vto 31/10 $30.388,66 · boleta AGIP PDF _inbox · sin pago MP aún</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="15" t="n">
+        <v>46339</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ABL — partida 1084069 · CUOTA 11/2026</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>28723</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>1084069</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>1084069 · ceil desde $28.722,26 · 1° vto 13/11/2026 · 2° vto 30/11 $30.935,65 · boleta AGIP PDF _inbox · sin pago MP aún</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="15" t="n">
+        <v>46370</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>ABL — partida 1084069 · CUOTA 12/2026</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>29556</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>1084069</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>1084069 · ceil desde $29.555,21 · 1° vto 14/12/2026 · 2° vto 31/12 $31.832,79 · boleta AGIP PDF _inbox · sin pago MP aún</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:J103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sync ABL AGIP debt and pending cuotas across all properties.
CIUDAD: overdue 08/09 at updated amounts, pending 10–12; reclassify Sep MP payment to BONORINO. OHIGGINS/BONORINO: load Oct–Dec pending boletas from ConsultaABL.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -742,10 +742,18 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
+      <c r="L7" s="5" t="n">
+        <v>27635</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>28215</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>28723</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>29556</v>
+      </c>
       <c r="P7" s="5">
         <f>SUM(D7:O7)</f>
         <v/>
@@ -1078,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2661,6 +2669,49 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="15" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ABL — partida 1084069 · CUOTA 09/2026</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>27635</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Dinero disponible</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>1084069</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>1084069 · ceil desde $27.634,08 · MP oficial 14/09/2026 · reclasificado desde CIUDAD (AGIP CIUDAD cuota 09 sigue VENCIDA; BONORINO 01-09 no aparecen como deuda → cuota 09 PAGADA)</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:J103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Align Edenor Chagas to BBVA cobro months; document Personal/Edesur Gmail gaps.
Reassign OHIGGINS Edenor Chagas (9267222037) by debit date from BBVA/Gmail,
place July from factura venc. 13/07, and mark Personal Feb/Mar/Ago plus Edesur
Jul as allowed empties when Gmail shows no separate cobro.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -1389,7 +1389,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Edesur</t>
+          <t>Edesur · cobro/venc. 03/08/2026</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Factura digital · vencimiento 03/08/2026 · cliente 3932799</t>
+          <t>Factura digital Gmail · emisión 21/07 · vencimiento 03/08/2026 · cliente 3932799</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Expensas BONORINO septiembre $226.137 (pago MP 10-oct)
Carga período septiembre (ceil desde $226.136,05) en Excel BONORINO
y espejo en Expensas Consorcios CIUDAD. MP dinero en cuenta.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/BONORINO/Gastos_BONORINO_2026.xlsx
+++ b/BONORINO/Gastos_BONORINO_2026.xlsx
@@ -666,7 +666,9 @@
         <v>209393</v>
       </c>
       <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
+      <c r="L5" s="5" t="n">
+        <v>226137</v>
+      </c>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="5" t="n"/>
@@ -1403,16 +1405,44 @@
       <c r="J10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="A11" s="9" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Expensas — Cons De Prop E Bonorino 82</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>226137</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Transferencia Mercado Pago</t>
+        </is>
+      </c>
       <c r="G11" s="10" t="n"/>
       <c r="H11" s="10" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Op 182412147771 · CUIT 30-53600400-5 · Banco Ciudad · CBU 0290018600000503750846 · Original 226136.05 · ceil · período septiembre 2026 · pago 10-oct · MP dinero en cuenta</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n"/>

</xml_diff>